<commit_message>
feat(transformations): paraleliza ajuste sazonal e organiza estrutura do projeto
- Adicionada função `seas_adj_parallel` em `seas_adj.py` utilizando `ThreadPoolExecutor` para acelerar o ajuste sazonal (X-13 ARIMA) em múltiplas séries simultaneamente. A função original `seas_adj` foi mantida para compatibilidade.
- Criada função auxiliar `_process_single_series` para isolar a chamada ao subprocesso do X-13.
- Correção do erro `X13NotFoundError` renomeando/duplicando o binário `x13as_ascii.exe` para `x13as.exe` na pasta x13as.
- Refatoração de diretório: movidos scripts obsoletos (`collect_data.py` e `main.py`) para a nova pasta `old/`.
- Correção de erros de digitação na coluna frequency (`Monhtly` -> `Monthly`) de variáveis automotivas no arquivo `series_spec.csv`.
- Adição de mais séries para o dataset
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -1,39 +1,74 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/741c46015d8d82fb/Documentos/PIB-Nowcast/pib_nowcast/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_085D1E5FD2616CEF6C7BC4B459C9D6BAAEBB8F6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5B87F71-C040-4547-92A7-0732323BFD0C}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="3795" yWindow="-12750" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+  <si>
+    <t>reference date</t>
+  </si>
+  <si>
+    <t>impacted variable</t>
+  </si>
+  <si>
+    <t>forecast</t>
+  </si>
+  <si>
+    <t>update_date</t>
+  </si>
+  <si>
+    <t>estimate</t>
+  </si>
+  <si>
+    <t>pib</t>
+  </si>
+  <si>
+    <t>predicted_mean</t>
+  </si>
+  <si>
+    <t>lower</t>
+  </si>
+  <si>
+    <t>upper</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -52,82 +87,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -415,102 +391,83 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>reference date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>impacted variable</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>update_date</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
         <v>46174</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>pib</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2.008346194886446</v>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>2.0083461948864461</v>
+      </c>
+      <c r="D2" s="2">
         <v>46197</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>predicted_mean</t>
-        </is>
+      <c r="E2" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
         <v>46174</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>pib</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>-2.02087055520173</v>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>-2.0208705552017299</v>
+      </c>
+      <c r="D3" s="2">
         <v>46197</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>lower</t>
-        </is>
+      <c r="E3" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>46174</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>pib</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>6.037562944974622</v>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>6.0375629449746224</v>
+      </c>
+      <c r="D4" s="2">
         <v>46197</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>upper</t>
-        </is>
+      <c r="E4" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: integra previsões de Índice e YoY% no pipeline do PIB
- Atualiza pipeline.py para usar ajuste sazonal STL paralelo
- Extrai e passa os fatores (factors) explicitamente na estimação do modelo DynamicFactorMQ
- Isola a série histórica de número-índice do PIB e calcula dinamicamente a data do próximo trimestre
- Atualiza `get_new_forecasts` em news.py para reconstruir matematicamente as previsões do Índice de Volume do PIB e das variações YoY% com base nos resultados de QoQ%
- Expande o arquivo de saída `forecasts.xlsx` para persistir os novos cálculos e seus intervalos de confiança
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -1,74 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/741c46015d8d82fb/Documentos/PIB-Nowcast/pib_nowcast/data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_085D1E5FD2616CEF6C7BC4B459C9D6BAAEBB8F6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5B87F71-C040-4547-92A7-0732323BFD0C}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="3795" yWindow="-12750" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
-  <si>
-    <t>reference date</t>
-  </si>
-  <si>
-    <t>impacted variable</t>
-  </si>
-  <si>
-    <t>forecast</t>
-  </si>
-  <si>
-    <t>update_date</t>
-  </si>
-  <si>
-    <t>estimate</t>
-  </si>
-  <si>
-    <t>pib</t>
-  </si>
-  <si>
-    <t>predicted_mean</t>
-  </si>
-  <si>
-    <t>lower</t>
-  </si>
-  <si>
-    <t>upper</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -87,23 +52,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -391,83 +415,422 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>46174</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>2.0083461948864461</v>
-      </c>
-      <c r="D2" s="2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>reference date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>impacted variable</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>update_date</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2.008346194886446</v>
+      </c>
+      <c r="D2" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="E2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <v>46174</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>-2.0208705552017299</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>-2.02087055520173</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="E3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>46174</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>6.0375629449746224</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6.037562944974622</v>
+      </c>
+      <c r="D4" s="1" t="n">
         <v>46197</v>
       </c>
-      <c r="E4" t="s">
-        <v>8</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.9167353008122705</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>-4.122703463224348</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5.964694657909964</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.9167353008122705</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>-4.122703463224348</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5.964694657909964</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>196.3133251806701</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>186.5101049529897</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>206.1331205180323</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5806564098115086</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>-4.441999716677081</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5.611804753577343</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add more series to spec
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1313,7 +1313,7 @@
       <c r="C35" t="n">
         <v>2.361475527766994</v>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="D35" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E35" t="inlineStr">
@@ -1339,7 +1339,7 @@
       <c r="C36" t="n">
         <v>0.2862643557493856</v>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E36" t="inlineStr">
@@ -1365,7 +1365,7 @@
       <c r="C37" t="n">
         <v>4.390495102402518</v>
       </c>
-      <c r="D37" s="2" t="n">
+      <c r="D37" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E37" t="inlineStr">
@@ -1391,7 +1391,7 @@
       <c r="C38" t="n">
         <v>199.1237783441651</v>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="D38" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E38" t="inlineStr">
@@ -1417,7 +1417,7 @@
       <c r="C39" t="n">
         <v>195.0868700512393</v>
       </c>
-      <c r="D39" s="2" t="n">
+      <c r="D39" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E39" t="inlineStr">
@@ -1443,7 +1443,7 @@
       <c r="C40" t="n">
         <v>203.0708301227036</v>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="D40" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E40" t="inlineStr">
@@ -1469,7 +1469,7 @@
       <c r="C41" t="n">
         <v>2.020585277264653</v>
       </c>
-      <c r="D41" s="2" t="n">
+      <c r="D41" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E41" t="inlineStr">
@@ -1495,7 +1495,7 @@
       <c r="C42" t="n">
         <v>-0.047714903556062</v>
       </c>
-      <c r="D42" s="2" t="n">
+      <c r="D42" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E42" t="inlineStr">
@@ -1521,7 +1521,7 @@
       <c r="C43" t="n">
         <v>4.042847690697626</v>
       </c>
-      <c r="D43" s="2" t="n">
+      <c r="D43" s="1" t="n">
         <v>46209</v>
       </c>
       <c r="E43" t="inlineStr">
@@ -1530,6 +1530,240 @@
         </is>
       </c>
       <c r="F43" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2.361819784643235</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>0.2863594682021482</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4.390590214855258</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>199.1244480270665</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>195.0870550734936</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>203.071015144958</v>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2.020928387676224</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>-0.04762010785241966</v>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>4.042942486401246</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
         <is>
           <t>yoy</t>
         </is>

</xml_diff>

<commit_message>
Create feats. an dhanges on model creation
* (feat) add `deflate` function to address nominal variables

* (spec) add new data

* (spec) add new factor block, Credit
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1547,7 +1547,7 @@
       <c r="C44" t="n">
         <v>2.361819784643235</v>
       </c>
-      <c r="D44" s="2" t="n">
+      <c r="D44" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E44" t="inlineStr">
@@ -1573,7 +1573,7 @@
       <c r="C45" t="n">
         <v>0.2863594682021482</v>
       </c>
-      <c r="D45" s="2" t="n">
+      <c r="D45" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E45" t="inlineStr">
@@ -1599,7 +1599,7 @@
       <c r="C46" t="n">
         <v>4.390590214855258</v>
       </c>
-      <c r="D46" s="2" t="n">
+      <c r="D46" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E46" t="inlineStr">
@@ -1625,7 +1625,7 @@
       <c r="C47" t="n">
         <v>199.1244480270665</v>
       </c>
-      <c r="D47" s="2" t="n">
+      <c r="D47" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E47" t="inlineStr">
@@ -1651,7 +1651,7 @@
       <c r="C48" t="n">
         <v>195.0870550734936</v>
       </c>
-      <c r="D48" s="2" t="n">
+      <c r="D48" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E48" t="inlineStr">
@@ -1677,7 +1677,7 @@
       <c r="C49" t="n">
         <v>203.071015144958</v>
       </c>
-      <c r="D49" s="2" t="n">
+      <c r="D49" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E49" t="inlineStr">
@@ -1703,7 +1703,7 @@
       <c r="C50" t="n">
         <v>2.020928387676224</v>
       </c>
-      <c r="D50" s="2" t="n">
+      <c r="D50" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E50" t="inlineStr">
@@ -1729,7 +1729,7 @@
       <c r="C51" t="n">
         <v>-0.04762010785241966</v>
       </c>
-      <c r="D51" s="2" t="n">
+      <c r="D51" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E51" t="inlineStr">
@@ -1755,7 +1755,7 @@
       <c r="C52" t="n">
         <v>4.042942486401246</v>
       </c>
-      <c r="D52" s="2" t="n">
+      <c r="D52" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="E52" t="inlineStr">
@@ -1764,6 +1764,942 @@
         </is>
       </c>
       <c r="F52" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2.233652828418463</v>
+      </c>
+      <c r="D53" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>0.1718096256754698</v>
+      </c>
+      <c r="D54" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>4.334326367528936</v>
+      </c>
+      <c r="D55" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>198.8751248471224</v>
+      </c>
+      <c r="D56" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>194.8642212648265</v>
+      </c>
+      <c r="D57" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>202.961565082754</v>
+      </c>
+      <c r="D58" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>1.893188260642686</v>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>-0.1617884697066918</v>
+      </c>
+      <c r="D60" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>3.986866012272783</v>
+      </c>
+      <c r="D61" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2.224490766530104</v>
+      </c>
+      <c r="D62" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>0.2337222726383241</v>
+      </c>
+      <c r="D63" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>4.251578895986178</v>
+      </c>
+      <c r="D64" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>198.857301888131</v>
+      </c>
+      <c r="D65" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>194.9846599369633</v>
+      </c>
+      <c r="D66" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>202.8005964263619</v>
+      </c>
+      <c r="D67" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1.884056710795678</v>
+      </c>
+      <c r="D68" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>-0.1000820079089526</v>
+      </c>
+      <c r="D69" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>3.904394111262377</v>
+      </c>
+      <c r="D70" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>2.29182348707293</v>
+      </c>
+      <c r="D71" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>0.2693580524859449</v>
+      </c>
+      <c r="D72" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>4.321498157783827</v>
+      </c>
+      <c r="D73" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>198.988284229403</v>
+      </c>
+      <c r="D74" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>195.0539822195009</v>
+      </c>
+      <c r="D75" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>202.9366103663369</v>
+      </c>
+      <c r="D76" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>1.951165195923243</v>
+      </c>
+      <c r="D77" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>-0.06456490444672891</v>
+      </c>
+      <c r="D78" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>3.974080523791823</v>
+      </c>
+      <c r="D79" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>2.291812295264857</v>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>0.2693385203149146</v>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>4.321493071811869</v>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>198.9882624579787</v>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>195.0539442235686</v>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>202.9366004725956</v>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1.951154041386771</v>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>-0.06458437157055297</v>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>3.974075454757453</v>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
         <is>
           <t>yoy</t>
         </is>

</xml_diff>

<commit_message>
add new series, simplify model specification
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2483,7 +2483,7 @@
       <c r="C80" t="n">
         <v>2.291812295264857</v>
       </c>
-      <c r="D80" s="2" t="n">
+      <c r="D80" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E80" t="inlineStr">
@@ -2509,7 +2509,7 @@
       <c r="C81" t="n">
         <v>0.2693385203149146</v>
       </c>
-      <c r="D81" s="2" t="n">
+      <c r="D81" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E81" t="inlineStr">
@@ -2535,7 +2535,7 @@
       <c r="C82" t="n">
         <v>4.321493071811869</v>
       </c>
-      <c r="D82" s="2" t="n">
+      <c r="D82" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E82" t="inlineStr">
@@ -2561,7 +2561,7 @@
       <c r="C83" t="n">
         <v>198.9882624579787</v>
       </c>
-      <c r="D83" s="2" t="n">
+      <c r="D83" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E83" t="inlineStr">
@@ -2587,7 +2587,7 @@
       <c r="C84" t="n">
         <v>195.0539442235686</v>
       </c>
-      <c r="D84" s="2" t="n">
+      <c r="D84" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E84" t="inlineStr">
@@ -2613,7 +2613,7 @@
       <c r="C85" t="n">
         <v>202.9366004725956</v>
       </c>
-      <c r="D85" s="2" t="n">
+      <c r="D85" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E85" t="inlineStr">
@@ -2639,7 +2639,7 @@
       <c r="C86" t="n">
         <v>1.951154041386771</v>
       </c>
-      <c r="D86" s="2" t="n">
+      <c r="D86" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E86" t="inlineStr">
@@ -2665,7 +2665,7 @@
       <c r="C87" t="n">
         <v>-0.06458437157055297</v>
       </c>
-      <c r="D87" s="2" t="n">
+      <c r="D87" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E87" t="inlineStr">
@@ -2691,7 +2691,7 @@
       <c r="C88" t="n">
         <v>3.974075454757453</v>
       </c>
-      <c r="D88" s="2" t="n">
+      <c r="D88" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="E88" t="inlineStr">
@@ -2700,6 +2700,240 @@
         </is>
       </c>
       <c r="F88" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>2.090993608449448</v>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>0.05537648863321687</v>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>4.086998780621833</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>198.5976098665167</v>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>194.6377238833382</v>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>202.4804387279437</v>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>1.75100413286029</v>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>-0.2778338542175574</v>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>3.740362090349247</v>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
         <is>
           <t>yoy</t>
         </is>

</xml_diff>

<commit_message>
more pipe, change to monthly, extract factors
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2717,7 +2717,7 @@
       <c r="C89" t="n">
         <v>2.090993608449448</v>
       </c>
-      <c r="D89" s="2" t="n">
+      <c r="D89" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E89" t="inlineStr">
@@ -2743,7 +2743,7 @@
       <c r="C90" t="n">
         <v>0.05537648863321687</v>
       </c>
-      <c r="D90" s="2" t="n">
+      <c r="D90" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E90" t="inlineStr">
@@ -2769,7 +2769,7 @@
       <c r="C91" t="n">
         <v>4.086998780621833</v>
       </c>
-      <c r="D91" s="2" t="n">
+      <c r="D91" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E91" t="inlineStr">
@@ -2795,7 +2795,7 @@
       <c r="C92" t="n">
         <v>198.5976098665167</v>
       </c>
-      <c r="D92" s="2" t="n">
+      <c r="D92" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E92" t="inlineStr">
@@ -2821,7 +2821,7 @@
       <c r="C93" t="n">
         <v>194.6377238833382</v>
       </c>
-      <c r="D93" s="2" t="n">
+      <c r="D93" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E93" t="inlineStr">
@@ -2847,7 +2847,7 @@
       <c r="C94" t="n">
         <v>202.4804387279437</v>
       </c>
-      <c r="D94" s="2" t="n">
+      <c r="D94" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E94" t="inlineStr">
@@ -2873,7 +2873,7 @@
       <c r="C95" t="n">
         <v>1.75100413286029</v>
       </c>
-      <c r="D95" s="2" t="n">
+      <c r="D95" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E95" t="inlineStr">
@@ -2899,7 +2899,7 @@
       <c r="C96" t="n">
         <v>-0.2778338542175574</v>
       </c>
-      <c r="D96" s="2" t="n">
+      <c r="D96" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E96" t="inlineStr">
@@ -2925,7 +2925,7 @@
       <c r="C97" t="n">
         <v>3.740362090349247</v>
       </c>
-      <c r="D97" s="2" t="n">
+      <c r="D97" s="1" t="n">
         <v>46218</v>
       </c>
       <c r="E97" t="inlineStr">
@@ -2934,6 +2934,708 @@
         </is>
       </c>
       <c r="F97" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>2.046580855023096</v>
+      </c>
+      <c r="D98" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>0.05417225737191345</v>
+      </c>
+      <c r="D99" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>4.027702472809297</v>
+      </c>
+      <c r="D100" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>198.5112137372764</v>
+      </c>
+      <c r="D101" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>194.6353812922656</v>
+      </c>
+      <c r="D102" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>202.3650896203559</v>
+      </c>
+      <c r="D103" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>1.706739285416758</v>
+      </c>
+      <c r="D104" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>-0.2790340750765452</v>
+      </c>
+      <c r="D105" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>3.681263254614175</v>
+      </c>
+      <c r="D106" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>2.139892828602843</v>
+      </c>
+      <c r="D107" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>-2.019490735844413</v>
+      </c>
+      <c r="D108" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>6.198600573975947</v>
+      </c>
+      <c r="D109" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>198.6927335194811</v>
+      </c>
+      <c r="D110" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>190.6014846715619</v>
+      </c>
+      <c r="D111" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>206.5881376965554</v>
+      </c>
+      <c r="D112" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1.799740505933567</v>
+      </c>
+      <c r="D113" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>-2.345791232932748</v>
+      </c>
+      <c r="D114" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>5.844931702303202</v>
+      </c>
+      <c r="D115" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>2.139892828602843</v>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>-2.019490735844413</v>
+      </c>
+      <c r="D117" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>6.198600573975947</v>
+      </c>
+      <c r="D118" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>198.6927335194811</v>
+      </c>
+      <c r="D119" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>190.6014846715619</v>
+      </c>
+      <c r="D120" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>206.5881376965554</v>
+      </c>
+      <c r="D121" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1.799740505933567</v>
+      </c>
+      <c r="D122" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>-2.345791232932748</v>
+      </c>
+      <c r="D123" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>5.844931702303202</v>
+      </c>
+      <c r="D124" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
         <is>
           <t>yoy</t>
         </is>

</xml_diff>

<commit_message>
Avança no EDA de fatores, algumas runs
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -701,7 +701,7 @@
       <c r="C11" t="n">
         <v>2.297004686936556</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -727,7 +727,7 @@
       <c r="C12" t="n">
         <v>0.5019356399627948</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -753,7 +753,7 @@
       <c r="C13" t="n">
         <v>4.127440306531241</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E13" t="inlineStr">
@@ -779,7 +779,7 @@
       <c r="C14" t="n">
         <v>198.9983632174977</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -805,7 +805,7 @@
       <c r="C15" t="n">
         <v>195.5064154004196</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -831,7 +831,7 @@
       <c r="C16" t="n">
         <v>202.5591096282952</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -857,7 +857,7 @@
       <c r="C17" t="n">
         <v>1.956329141048108</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E17" t="inlineStr">
@@ -883,7 +883,7 @@
       <c r="C18" t="n">
         <v>0.1672381393685862</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E18" t="inlineStr">
@@ -909,7 +909,7 @@
       <c r="C19" t="n">
         <v>3.780668935493003</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E19" t="inlineStr">
@@ -918,6 +918,240 @@
         </is>
       </c>
       <c r="F19" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2.298445817988515</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.502583126444397</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>4.128087794125442</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>199.0011666497331</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>195.5076749558723</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>202.5603691859122</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1.957765472760054</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.1678834695523435</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3.781314266785629</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>yoy</t>
         </is>

</xml_diff>

<commit_message>
Algumas runs e novas funções de news
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,7 +935,7 @@
       <c r="C20" t="n">
         <v>2.298445817988515</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E20" t="inlineStr">
@@ -961,7 +961,7 @@
       <c r="C21" t="n">
         <v>0.502583126444397</v>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E21" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="C22" t="n">
         <v>4.128087794125442</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E22" t="inlineStr">
@@ -1013,7 +1013,7 @@
       <c r="C23" t="n">
         <v>199.0011666497331</v>
       </c>
-      <c r="D23" s="2" t="n">
+      <c r="D23" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E23" t="inlineStr">
@@ -1039,7 +1039,7 @@
       <c r="C24" t="n">
         <v>195.5076749558723</v>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E24" t="inlineStr">
@@ -1065,7 +1065,7 @@
       <c r="C25" t="n">
         <v>202.5603691859122</v>
       </c>
-      <c r="D25" s="2" t="n">
+      <c r="D25" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E25" t="inlineStr">
@@ -1091,7 +1091,7 @@
       <c r="C26" t="n">
         <v>1.957765472760054</v>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E26" t="inlineStr">
@@ -1117,7 +1117,7 @@
       <c r="C27" t="n">
         <v>0.1678834695523435</v>
       </c>
-      <c r="D27" s="2" t="n">
+      <c r="D27" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E27" t="inlineStr">
@@ -1143,7 +1143,7 @@
       <c r="C28" t="n">
         <v>3.781314266785629</v>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="D28" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="E28" t="inlineStr">
@@ -1152,6 +1152,240 @@
         </is>
       </c>
       <c r="F28" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1.974175046073926</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>-0.06428154736655411</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4.181452730033903</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>198.3703627171276</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>194.4049531059079</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>202.6641799957349</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1.634574606582451</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>-0.3970933979363434</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3.834501483622765</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>yoy</t>
         </is>

</xml_diff>

<commit_message>
feat: Ajustar modelo DFM para série mensal com novos parâmetros
- Alterar fonte de dados de série anual para mensal
- Mudar data inicial de fit para 2002-01-01 (antes era 2005-01-01)
- Atualizar fator Global de multiplicidade 2 para 4
- Remover 'Sentiment' dos fatores de ordem
- Ajustar k_endog_monthly reduzindo em 1
- Adicionar análises de diagnóstico (coeficientes de determinação e plots de diagnóstico)
- Configurar arquivo de dados dinâmico baseado em tipo de série (MONTHLY/ANNUAL)
- Atualizar arquivos de especificação e parâmetros do modelo
</commit_message>
<xml_diff>
--- a/pib_nowcast/data/forecasts.xlsx
+++ b/pib_nowcast/data/forecasts.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1444,7 +1444,7 @@
       <c r="C38" t="n">
         <v>1.841392547013983</v>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="D38" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="E38" t="inlineStr">
@@ -1467,7 +1467,7 @@
       <c r="C39" t="n">
         <v>0.2281087881378294</v>
       </c>
-      <c r="D39" s="2" t="n">
+      <c r="D39" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="E39" t="inlineStr">
@@ -1494,7 +1494,7 @@
       <c r="C40" t="n">
         <v>4.016321610490387</v>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="D40" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="E40" t="inlineStr">
@@ -1512,6 +1512,1464 @@
           <t>pib</t>
         </is>
       </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>4.21177176982699</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>-17.42362082929858</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>21.46667085238697</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>202.7231596238445</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>160.6358304007655</v>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>236.2891148091483</v>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>3.864719553153217</v>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>-17.69862157968774</v>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>21.06215534847236</v>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1.192683245269823</v>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>-7.001251551511965</v>
+      </c>
+      <c r="D51" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>11.28814918296648</v>
+      </c>
+      <c r="D52" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>199.6936411162155</v>
+      </c>
+      <c r="D53" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>183.5237301882463</v>
+      </c>
+      <c r="D54" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>219.616033597666</v>
+      </c>
+      <c r="D55" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2.670252501910264</v>
+      </c>
+      <c r="D56" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>-5.643326381364377</v>
+      </c>
+      <c r="D57" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>12.91312781371006</v>
+      </c>
+      <c r="D58" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>0.5017162721947411</v>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>-0.6174935364728439</v>
+      </c>
+      <c r="D60" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2.020520681210353</v>
+      </c>
+      <c r="D61" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>198.3300868915491</v>
+      </c>
+      <c r="D62" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>196.1214382551245</v>
+      </c>
+      <c r="D63" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>201.3272955123005</v>
+      </c>
+      <c r="D64" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1.969196345269464</v>
+      </c>
+      <c r="D65" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>0.8336443471077093</v>
+      </c>
+      <c r="D66" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>3.510177641285606</v>
+      </c>
+      <c r="D67" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2.084533021488257</v>
+      </c>
+      <c r="D68" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>-2.233477386927855</v>
+      </c>
+      <c r="D69" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>8.285057790919765</v>
+      </c>
+      <c r="D70" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>201.4536174646049</v>
+      </c>
+      <c r="D71" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>192.9324557246366</v>
+      </c>
+      <c r="D72" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>213.6897330446011</v>
+      </c>
+      <c r="D73" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>3.575124660465256</v>
+      </c>
+      <c r="D74" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>-0.8059353600840202</v>
+      </c>
+      <c r="D75" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>9.866186655321885</v>
+      </c>
+      <c r="D76" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>2.091223890401314</v>
+      </c>
+      <c r="D77" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>-2.149056712392478</v>
+      </c>
+      <c r="D78" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>8.353494259094031</v>
+      </c>
+      <c r="D79" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>201.4668212253179</v>
+      </c>
+      <c r="D80" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>193.0990514837647</v>
+      </c>
+      <c r="D81" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>213.8247855708962</v>
+      </c>
+      <c r="D82" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>3.581913226384548</v>
+      </c>
+      <c r="D83" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>-0.7202820134886045</v>
+      </c>
+      <c r="D84" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>9.935622401489042</v>
+      </c>
+      <c r="D85" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>2.242868034165349</v>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>-2.20396162863261</v>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>8.445180158653836</v>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>qoq</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>201.7660757786219</v>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>192.9907021220564</v>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>214.0057185250875</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>3.735771608545968</v>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>predicted_mean</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>-0.7759886261920812</v>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>10.02864705660025</v>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>yoy</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>